<commit_message>
Fix IdealWornArea: use EdgeRadius^2*C not full-mask Apollonius solver
The Apollonius solver on the full tool body mask placed P at the image
far corner (~800px from origin), giving r~250px and area~20000px^2.
Correct formula: r^2 * (cot40 - (pi/2 - 40rad)) using RANSAC edge radius
(2-17px) giving IdealWornArea range 1.3-93 px^2. Excel recomputed.
Python fallback also reverted to fast formula.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestData/Tool_Features_Dataset.xlsx
+++ b/TestData/Tool_Features_Dataset.xlsx
@@ -467,7 +467,7 @@
         <v>310</v>
       </c>
       <c r="F2" t="n">
-        <v>20870.90456199991</v>
+        <v>2.439920371617494</v>
       </c>
     </row>
     <row r="3">
@@ -489,7 +489,7 @@
         <v>294</v>
       </c>
       <c r="F3" t="n">
-        <v>17981.51323683338</v>
+        <v>27.10970732889851</v>
       </c>
     </row>
     <row r="4">
@@ -511,7 +511,7 @@
         <v>743</v>
       </c>
       <c r="F4" t="n">
-        <v>19321.85079992714</v>
+        <v>32.15407371083133</v>
       </c>
     </row>
     <row r="5">
@@ -533,7 +533,7 @@
         <v>854</v>
       </c>
       <c r="F5" t="n">
-        <v>20145.78489556805</v>
+        <v>6.377524170087523</v>
       </c>
     </row>
     <row r="6">
@@ -555,7 +555,7 @@
         <v>930</v>
       </c>
       <c r="F6" t="n">
-        <v>14526.91091007684</v>
+        <v>16.38882677143986</v>
       </c>
     </row>
     <row r="7">
@@ -577,7 +577,7 @@
         <v>2115</v>
       </c>
       <c r="F7" t="n">
-        <v>20206.24772210317</v>
+        <v>46.12204719511584</v>
       </c>
     </row>
     <row r="8">
@@ -599,7 +599,7 @@
         <v>2809</v>
       </c>
       <c r="F8" t="n">
-        <v>16234.77973440828</v>
+        <v>23.04551878021796</v>
       </c>
     </row>
     <row r="9">
@@ -621,7 +621,7 @@
         <v>672</v>
       </c>
       <c r="F9" t="n">
-        <v>19504.29837802124</v>
+        <v>22.89371284992501</v>
       </c>
     </row>
     <row r="10">
@@ -643,7 +643,7 @@
         <v>502</v>
       </c>
       <c r="F10" t="n">
-        <v>20074.60934410752</v>
+        <v>13.42239955260406</v>
       </c>
     </row>
     <row r="11">
@@ -665,7 +665,7 @@
         <v>1300</v>
       </c>
       <c r="F11" t="n">
-        <v>18686.19961344027</v>
+        <v>10.03639299153215</v>
       </c>
     </row>
     <row r="12">
@@ -687,7 +687,7 @@
         <v>1041</v>
       </c>
       <c r="F12" t="n">
-        <v>21957.87754470446</v>
+        <v>11.49360188671716</v>
       </c>
     </row>
     <row r="13">
@@ -709,7 +709,7 @@
         <v>1006</v>
       </c>
       <c r="F13" t="n">
-        <v>19864.36608254952</v>
+        <v>92.99893100894592</v>
       </c>
     </row>
     <row r="14">
@@ -731,7 +731,7 @@
         <v>1050</v>
       </c>
       <c r="F14" t="n">
-        <v>17531.51135954081</v>
+        <v>55.61727051939595</v>
       </c>
     </row>
     <row r="15">
@@ -753,7 +753,7 @@
         <v>790</v>
       </c>
       <c r="F15" t="n">
-        <v>21514.90719960774</v>
+        <v>14.14880064744904</v>
       </c>
     </row>
     <row r="16">
@@ -775,7 +775,7 @@
         <v>986</v>
       </c>
       <c r="F16" t="n">
-        <v>20648.83604287046</v>
+        <v>10.88168591171883</v>
       </c>
     </row>
     <row r="17">
@@ -797,7 +797,7 @@
         <v>910</v>
       </c>
       <c r="F17" t="n">
-        <v>21979.97205675448</v>
+        <v>7.846748419471045</v>
       </c>
     </row>
     <row r="18">
@@ -819,7 +819,7 @@
         <v>881</v>
       </c>
       <c r="F18" t="n">
-        <v>21871.70351482536</v>
+        <v>7.085169428140403</v>
       </c>
     </row>
     <row r="19">
@@ -841,7 +841,7 @@
         <v>1374</v>
       </c>
       <c r="F19" t="n">
-        <v>22333.14272613524</v>
+        <v>6.935111220188841</v>
       </c>
     </row>
     <row r="20">
@@ -863,7 +863,7 @@
         <v>1144</v>
       </c>
       <c r="F20" t="n">
-        <v>19894.51797377082</v>
+        <v>28.18326462925183</v>
       </c>
     </row>
     <row r="21">
@@ -885,7 +885,7 @@
         <v>6374</v>
       </c>
       <c r="F21" t="n">
-        <v>16382.88950886733</v>
+        <v>18.99784832799481</v>
       </c>
     </row>
     <row r="22">
@@ -907,7 +907,7 @@
         <v>1426</v>
       </c>
       <c r="F22" t="n">
-        <v>18448.05257016527</v>
+        <v>23.72483496851398</v>
       </c>
     </row>
     <row r="23">
@@ -929,7 +929,7 @@
         <v>1488</v>
       </c>
       <c r="F23" t="n">
-        <v>18913.31198875631</v>
+        <v>4.879474306958572</v>
       </c>
     </row>
     <row r="24">
@@ -951,7 +951,7 @@
         <v>1232</v>
       </c>
       <c r="F24" t="n">
-        <v>18146.97267879952</v>
+        <v>12.95220488318765</v>
       </c>
     </row>
     <row r="25">
@@ -973,7 +973,7 @@
         <v>1257</v>
       </c>
       <c r="F25" t="n">
-        <v>16976.60914600706</v>
+        <v>21.67036706688243</v>
       </c>
     </row>
     <row r="26">
@@ -995,7 +995,7 @@
         <v>1084</v>
       </c>
       <c r="F26" t="n">
-        <v>20376.51645899115</v>
+        <v>4.503377652657182</v>
       </c>
     </row>
     <row r="27">
@@ -1017,7 +1017,7 @@
         <v>1198</v>
       </c>
       <c r="F27" t="n">
-        <v>20705.90767166334</v>
+        <v>20.37339769766294</v>
       </c>
     </row>
     <row r="28">
@@ -1039,7 +1039,7 @@
         <v>1391</v>
       </c>
       <c r="F28" t="n">
-        <v>20796.96252417873</v>
+        <v>1.697549485432904</v>
       </c>
     </row>
     <row r="29">
@@ -1061,7 +1061,7 @@
         <v>1351</v>
       </c>
       <c r="F29" t="n">
-        <v>19701.39728198577</v>
+        <v>1.589006169446293</v>
       </c>
     </row>
     <row r="30">
@@ -1083,7 +1083,7 @@
         <v>1179</v>
       </c>
       <c r="F30" t="n">
-        <v>20204.03238109461</v>
+        <v>4.216821369245362</v>
       </c>
     </row>
     <row r="31">
@@ -1105,7 +1105,7 @@
         <v>4807</v>
       </c>
       <c r="F31" t="n">
-        <v>21980.46972834383</v>
+        <v>6.217360115102863</v>
       </c>
     </row>
     <row r="32">
@@ -1127,7 +1127,7 @@
         <v>1931</v>
       </c>
       <c r="F32" t="n">
-        <v>21923.78123213959</v>
+        <v>20.23459363901321</v>
       </c>
     </row>
     <row r="33">
@@ -1149,7 +1149,7 @@
         <v>1896</v>
       </c>
       <c r="F33" t="n">
-        <v>21717.17175167283</v>
+        <v>21.3754936551423</v>
       </c>
     </row>
     <row r="34">
@@ -1171,7 +1171,7 @@
         <v>4313</v>
       </c>
       <c r="F34" t="n">
-        <v>21541.98724422756</v>
+        <v>12.35777415360895</v>
       </c>
     </row>
     <row r="35">
@@ -1193,7 +1193,7 @@
         <v>2904</v>
       </c>
       <c r="F35" t="n">
-        <v>21869.60314219038</v>
+        <v>15.0323490636261</v>
       </c>
     </row>
     <row r="36">
@@ -1215,7 +1215,7 @@
         <v>4219</v>
       </c>
       <c r="F36" t="n">
-        <v>21490.02133222659</v>
+        <v>14.15558418386924</v>
       </c>
     </row>
     <row r="37">
@@ -1237,7 +1237,7 @@
         <v>4933</v>
       </c>
       <c r="F37" t="n">
-        <v>21911.88354933208</v>
+        <v>8.31774478882752</v>
       </c>
     </row>
     <row r="38">
@@ -1259,7 +1259,7 @@
         <v>3124</v>
       </c>
       <c r="F38" t="n">
-        <v>21952.6903186737</v>
+        <v>8.055772137217547</v>
       </c>
     </row>
     <row r="39">
@@ -1281,7 +1281,7 @@
         <v>3140</v>
       </c>
       <c r="F39" t="n">
-        <v>21711.99914642012</v>
+        <v>7.980582934569238</v>
       </c>
     </row>
     <row r="40">
@@ -1303,7 +1303,7 @@
         <v>2424</v>
       </c>
       <c r="F40" t="n">
-        <v>21984.34299589061</v>
+        <v>8.001011473914865</v>
       </c>
     </row>
     <row r="41">
@@ -1325,7 +1325,7 @@
         <v>4495</v>
       </c>
       <c r="F41" t="n">
-        <v>22057.57158462311</v>
+        <v>8.812063314458051</v>
       </c>
     </row>
     <row r="42">
@@ -1347,7 +1347,7 @@
         <v>2447</v>
       </c>
       <c r="F42" t="n">
-        <v>22525.16702158202</v>
+        <v>17.13817924520275</v>
       </c>
     </row>
     <row r="43">
@@ -1369,7 +1369,7 @@
         <v>3105</v>
       </c>
       <c r="F43" t="n">
-        <v>22685.15642528117</v>
+        <v>10.30607265239863</v>
       </c>
     </row>
     <row r="44">
@@ -1391,7 +1391,7 @@
         <v>5051</v>
       </c>
       <c r="F44" t="n">
-        <v>22018.58720188544</v>
+        <v>12.75848668866579</v>
       </c>
     </row>
     <row r="45">
@@ -1413,7 +1413,7 @@
         <v>3801</v>
       </c>
       <c r="F45" t="n">
-        <v>22599.75986232793</v>
+        <v>13.52927971869998</v>
       </c>
     </row>
     <row r="46">
@@ -1435,7 +1435,7 @@
         <v>3358</v>
       </c>
       <c r="F46" t="n">
-        <v>22669.89860182178</v>
+        <v>6.608320033624201</v>
       </c>
     </row>
     <row r="47">
@@ -1457,7 +1457,7 @@
         <v>5613</v>
       </c>
       <c r="F47" t="n">
-        <v>23044.23861568442</v>
+        <v>14.10607705029087</v>
       </c>
     </row>
     <row r="48">
@@ -1479,7 +1479,7 @@
         <v>5679</v>
       </c>
       <c r="F48" t="n">
-        <v>23037.63616996561</v>
+        <v>12.19407528765311</v>
       </c>
     </row>
     <row r="49">
@@ -1501,7 +1501,7 @@
         <v>1785</v>
       </c>
       <c r="F49" t="n">
-        <v>23074.62588490692</v>
+        <v>6.597700093377101</v>
       </c>
     </row>
     <row r="50">
@@ -1523,7 +1523,7 @@
         <v>2637</v>
       </c>
       <c r="F50" t="n">
-        <v>22639.11958035273</v>
+        <v>41.39271211290123</v>
       </c>
     </row>
     <row r="51">
@@ -1545,7 +1545,7 @@
         <v>3744</v>
       </c>
       <c r="F51" t="n">
-        <v>22870.67089063587</v>
+        <v>22.15971178486427</v>
       </c>
     </row>
     <row r="52">
@@ -1567,7 +1567,7 @@
         <v>327</v>
       </c>
       <c r="F52" t="n">
-        <v>18603.05554248795</v>
+        <v>1.729296436897034</v>
       </c>
     </row>
     <row r="53">
@@ -1589,7 +1589,7 @@
         <v>223</v>
       </c>
       <c r="F53" t="n">
-        <v>16748.96240810622</v>
+        <v>17.18868987691263</v>
       </c>
     </row>
     <row r="54">
@@ -1611,7 +1611,7 @@
         <v>364</v>
       </c>
       <c r="F54" t="n">
-        <v>19259.96170465082</v>
+        <v>9.147255602972042</v>
       </c>
     </row>
     <row r="55">
@@ -1633,7 +1633,7 @@
         <v>5667</v>
       </c>
       <c r="F55" t="n">
-        <v>21814.91385751297</v>
+        <v>18.72251473474099</v>
       </c>
     </row>
     <row r="56">
@@ -1655,7 +1655,7 @@
         <v>3394</v>
       </c>
       <c r="F56" t="n">
-        <v>21803.26779528261</v>
+        <v>13.97762449386687</v>
       </c>
     </row>
     <row r="57">
@@ -1677,7 +1677,7 @@
         <v>3658</v>
       </c>
       <c r="F57" t="n">
-        <v>21647.75867861363</v>
+        <v>21.43183370709438</v>
       </c>
     </row>
     <row r="58">
@@ -1699,7 +1699,7 @@
         <v>6668</v>
       </c>
       <c r="F58" t="n">
-        <v>20588.34295655577</v>
+        <v>23.9415802485354</v>
       </c>
     </row>
     <row r="59">
@@ -1721,7 +1721,7 @@
         <v>2869</v>
       </c>
       <c r="F59" t="n">
-        <v>21840.20576379199</v>
+        <v>15.0655313195675</v>
       </c>
     </row>
     <row r="60">
@@ -1743,7 +1743,7 @@
         <v>5619</v>
       </c>
       <c r="F60" t="n">
-        <v>20661.2228273911</v>
+        <v>10.03886564360537</v>
       </c>
     </row>
     <row r="61">
@@ -1765,7 +1765,7 @@
         <v>2614</v>
       </c>
       <c r="F61" t="n">
-        <v>21011.73040380819</v>
+        <v>6.780488910254409</v>
       </c>
     </row>
     <row r="62">
@@ -1787,7 +1787,7 @@
         <v>3711</v>
       </c>
       <c r="F62" t="n">
-        <v>20815.48551638666</v>
+        <v>26.12986857070972</v>
       </c>
     </row>
     <row r="63">
@@ -1809,7 +1809,7 @@
         <v>5703</v>
       </c>
       <c r="F63" t="n">
-        <v>20880.38323897567</v>
+        <v>9.723205204875883</v>
       </c>
     </row>
     <row r="64">
@@ -1831,7 +1831,7 @@
         <v>5601</v>
       </c>
       <c r="F64" t="n">
-        <v>20713.37312203141</v>
+        <v>13.24326881170739</v>
       </c>
     </row>
     <row r="65">
@@ -1853,7 +1853,7 @@
         <v>4721</v>
       </c>
       <c r="F65" t="n">
-        <v>17265.63763979949</v>
+        <v>12.22842866815003</v>
       </c>
     </row>
     <row r="66">
@@ -1875,7 +1875,7 @@
         <v>4755</v>
       </c>
       <c r="F66" t="n">
-        <v>15665.39172243119</v>
+        <v>13.96699487819664</v>
       </c>
     </row>
     <row r="67">
@@ -1897,7 +1897,7 @@
         <v>5323</v>
       </c>
       <c r="F67" t="n">
-        <v>17575.70511603928</v>
+        <v>14.46807813821597</v>
       </c>
     </row>
     <row r="68">
@@ -1919,7 +1919,7 @@
         <v>5344</v>
       </c>
       <c r="F68" t="n">
-        <v>17215.89435310641</v>
+        <v>9.582903511475827</v>
       </c>
     </row>
     <row r="69">
@@ -1941,7 +1941,7 @@
         <v>2552</v>
       </c>
       <c r="F69" t="n">
-        <v>16926.93310838525</v>
+        <v>10.32252382047532</v>
       </c>
     </row>
     <row r="70">
@@ -1963,7 +1963,7 @@
         <v>5000</v>
       </c>
       <c r="F70" t="n">
-        <v>16362.52971857128</v>
+        <v>10.50713355438784</v>
       </c>
     </row>
     <row r="71">
@@ -1985,7 +1985,7 @@
         <v>6537</v>
       </c>
       <c r="F71" t="n">
-        <v>18140.48154181615</v>
+        <v>13.36776931172639</v>
       </c>
     </row>
     <row r="72">
@@ -2007,7 +2007,7 @@
         <v>2273</v>
       </c>
       <c r="F72" t="n">
-        <v>19453.15036688542</v>
+        <v>18.77827089733691</v>
       </c>
     </row>
     <row r="73">
@@ -2029,7 +2029,7 @@
         <v>6696</v>
       </c>
       <c r="F73" t="n">
-        <v>19150.42489901725</v>
+        <v>11.58103114672432</v>
       </c>
     </row>
     <row r="74">
@@ -2051,7 +2051,7 @@
         <v>1779</v>
       </c>
       <c r="F74" t="n">
-        <v>19559.10443677177</v>
+        <v>23.25256969273133</v>
       </c>
     </row>
     <row r="75">
@@ -2073,7 +2073,7 @@
         <v>4393</v>
       </c>
       <c r="F75" t="n">
-        <v>21312.73675555709</v>
+        <v>33.10264884872034</v>
       </c>
     </row>
     <row r="76">
@@ -2095,7 +2095,7 @@
         <v>322</v>
       </c>
       <c r="F76" t="n">
-        <v>23613.1087988269</v>
+        <v>45.4215737152983</v>
       </c>
     </row>
     <row r="77">
@@ -2117,7 +2117,7 @@
         <v>568</v>
       </c>
       <c r="F77" t="n">
-        <v>19439.86799182185</v>
+        <v>4.234543894213822</v>
       </c>
     </row>
     <row r="78">
@@ -2139,7 +2139,7 @@
         <v>617</v>
       </c>
       <c r="F78" t="n">
-        <v>18425.8150324889</v>
+        <v>31.23761496066274</v>
       </c>
     </row>
     <row r="79">
@@ -2161,7 +2161,7 @@
         <v>618</v>
       </c>
       <c r="F79" t="n">
-        <v>17174.98667590443</v>
+        <v>7.82198101088568</v>
       </c>
     </row>
     <row r="80">
@@ -2183,7 +2183,7 @@
         <v>4677</v>
       </c>
       <c r="F80" t="n">
-        <v>21073.70096895389</v>
+        <v>27.66577915850095</v>
       </c>
     </row>
     <row r="81">
@@ -2205,7 +2205,7 @@
         <v>2017</v>
       </c>
       <c r="F81" t="n">
-        <v>19155.84097084849</v>
+        <v>6.627738400301133</v>
       </c>
     </row>
     <row r="82">
@@ -2227,7 +2227,7 @@
         <v>5778</v>
       </c>
       <c r="F82" t="n">
-        <v>20151.49404963906</v>
+        <v>14.40701221134602</v>
       </c>
     </row>
     <row r="83">
@@ -2249,7 +2249,7 @@
         <v>5600</v>
       </c>
       <c r="F83" t="n">
-        <v>20761.05833225043</v>
+        <v>14.58307782253222</v>
       </c>
     </row>
     <row r="84">
@@ -2271,7 +2271,7 @@
         <v>1945</v>
       </c>
       <c r="F84" t="n">
-        <v>21587.34885029928</v>
+        <v>7.775679188560902</v>
       </c>
     </row>
     <row r="85">
@@ -2293,7 +2293,7 @@
         <v>665</v>
       </c>
       <c r="F85" t="n">
-        <v>20130.52704191955</v>
+        <v>36.10462699908605</v>
       </c>
     </row>
     <row r="86">
@@ -2315,7 +2315,7 @@
         <v>707</v>
       </c>
       <c r="F86" t="n">
-        <v>19282.45524702189</v>
+        <v>22.77327259898772</v>
       </c>
     </row>
     <row r="87">
@@ -2337,7 +2337,7 @@
         <v>730</v>
       </c>
       <c r="F87" t="n">
-        <v>18679.66748809793</v>
+        <v>5.457947534687663</v>
       </c>
     </row>
     <row r="88">
@@ -2359,7 +2359,7 @@
         <v>3080</v>
       </c>
       <c r="F88" t="n">
-        <v>20434.06438622999</v>
+        <v>7.560292088281518</v>
       </c>
     </row>
     <row r="89">
@@ -2381,7 +2381,7 @@
         <v>1412</v>
       </c>
       <c r="F89" t="n">
-        <v>19471.61541422229</v>
+        <v>36.87212275271453</v>
       </c>
     </row>
     <row r="90">
@@ -2403,7 +2403,7 @@
         <v>892</v>
       </c>
       <c r="F90" t="n">
-        <v>22653.13101753918</v>
+        <v>10.05313644213033</v>
       </c>
     </row>
     <row r="91">
@@ -2425,7 +2425,7 @@
         <v>3765</v>
       </c>
       <c r="F91" t="n">
-        <v>15354.98090912011</v>
+        <v>14.85728454530859</v>
       </c>
     </row>
     <row r="92">
@@ -2447,7 +2447,7 @@
         <v>6738</v>
       </c>
       <c r="F92" t="n">
-        <v>18676.33152612249</v>
+        <v>18.11258202359485</v>
       </c>
     </row>
     <row r="93">
@@ -2469,7 +2469,7 @@
         <v>6685</v>
       </c>
       <c r="F93" t="n">
-        <v>17996.77515708792</v>
+        <v>16.49942709169994</v>
       </c>
     </row>
     <row r="94">
@@ -2491,7 +2491,7 @@
         <v>4465</v>
       </c>
       <c r="F94" t="n">
-        <v>21401.80836475177</v>
+        <v>20.00365335263664</v>
       </c>
     </row>
     <row r="95">
@@ -2513,7 +2513,7 @@
         <v>3584</v>
       </c>
       <c r="F95" t="n">
-        <v>20381.775452703</v>
+        <v>60.34629880794461</v>
       </c>
     </row>
     <row r="96">
@@ -2535,7 +2535,7 @@
         <v>2145</v>
       </c>
       <c r="F96" t="n">
-        <v>20535.29348109918</v>
+        <v>33.29341539928724</v>
       </c>
     </row>
     <row r="97">
@@ -2557,7 +2557,7 @@
         <v>1953</v>
       </c>
       <c r="F97" t="n">
-        <v>19668.4939794105</v>
+        <v>33.81988753076752</v>
       </c>
     </row>
     <row r="98">
@@ -2579,7 +2579,7 @@
         <v>5760</v>
       </c>
       <c r="F98" t="n">
-        <v>15571.0848621376</v>
+        <v>9.471781602926113</v>
       </c>
     </row>
     <row r="99">
@@ -2601,7 +2601,7 @@
         <v>4396</v>
       </c>
       <c r="F99" t="n">
-        <v>21016.06420488282</v>
+        <v>30.78414238840744</v>
       </c>
     </row>
     <row r="100">
@@ -2623,7 +2623,7 @@
         <v>5635</v>
       </c>
       <c r="F100" t="n">
-        <v>18979.35050931901</v>
+        <v>18.56323164748131</v>
       </c>
     </row>
     <row r="101">
@@ -2645,7 +2645,7 @@
         <v>5577</v>
       </c>
       <c r="F101" t="n">
-        <v>19602.50345954622</v>
+        <v>17.7519799219473</v>
       </c>
     </row>
     <row r="102">
@@ -2667,7 +2667,7 @@
         <v>639</v>
       </c>
       <c r="F102" t="n">
-        <v>20432.71146009028</v>
+        <v>11.8172699123333</v>
       </c>
     </row>
     <row r="103">
@@ -2689,7 +2689,7 @@
         <v>1214</v>
       </c>
       <c r="F103" t="n">
-        <v>19686.73106187942</v>
+        <v>14.4068825909476</v>
       </c>
     </row>
     <row r="104">
@@ -2711,7 +2711,7 @@
         <v>541</v>
       </c>
       <c r="F104" t="n">
-        <v>19665.00262206752</v>
+        <v>3.557074402416895</v>
       </c>
     </row>
     <row r="105">
@@ -2733,7 +2733,7 @@
         <v>667</v>
       </c>
       <c r="F105" t="n">
-        <v>21830.1944580236</v>
+        <v>14.1153686179375</v>
       </c>
     </row>
     <row r="106">
@@ -2755,7 +2755,7 @@
         <v>119</v>
       </c>
       <c r="F106" t="n">
-        <v>24316.04602364474</v>
+        <v>60.43462595267156</v>
       </c>
     </row>
     <row r="107">
@@ -2777,7 +2777,7 @@
         <v>86</v>
       </c>
       <c r="F107" t="n">
-        <v>23168.30427118813</v>
+        <v>7.319714378515583</v>
       </c>
     </row>
     <row r="108">
@@ -2799,7 +2799,7 @@
         <v>10</v>
       </c>
       <c r="F108" t="n">
-        <v>15793.31380216282</v>
+        <v>49.34021349046505</v>
       </c>
     </row>
     <row r="109">
@@ -2821,7 +2821,7 @@
         <v>883</v>
       </c>
       <c r="F109" t="n">
-        <v>19728.41490642258</v>
+        <v>1.288819738859011</v>
       </c>
     </row>
     <row r="110">
@@ -2843,7 +2843,7 @@
         <v>558</v>
       </c>
       <c r="F110" t="n">
-        <v>25002.59387600629</v>
+        <v>30.16513035374453</v>
       </c>
     </row>
     <row r="111">
@@ -2865,7 +2865,7 @@
         <v>632</v>
       </c>
       <c r="F111" t="n">
-        <v>19666.73580596706</v>
+        <v>8.067824239633536</v>
       </c>
     </row>
     <row r="112">
@@ -2887,7 +2887,7 @@
         <v>782</v>
       </c>
       <c r="F112" t="n">
-        <v>19472.80836498955</v>
+        <v>11.37018345809946</v>
       </c>
     </row>
     <row r="113">
@@ -2909,7 +2909,7 @@
         <v>984</v>
       </c>
       <c r="F113" t="n">
-        <v>18686.5817220923</v>
+        <v>33.20241654646102</v>
       </c>
     </row>
     <row r="114">
@@ -2931,7 +2931,7 @@
         <v>233</v>
       </c>
       <c r="F114" t="n">
-        <v>20115.46153809511</v>
+        <v>3.877367116413661</v>
       </c>
     </row>
     <row r="115">
@@ -2953,7 +2953,7 @@
         <v>1583</v>
       </c>
       <c r="F115" t="n">
-        <v>17733.1599989204</v>
+        <v>1.727969574417555</v>
       </c>
     </row>
     <row r="116">
@@ -2975,7 +2975,7 @@
         <v>1433</v>
       </c>
       <c r="F116" t="n">
-        <v>17320.55143256178</v>
+        <v>22.22703933695077</v>
       </c>
     </row>
     <row r="117">
@@ -2997,7 +2997,7 @@
         <v>893</v>
       </c>
       <c r="F117" t="n">
-        <v>20370.70210606915</v>
+        <v>5.698726990933433</v>
       </c>
     </row>
     <row r="118">
@@ -3019,7 +3019,7 @@
         <v>1062</v>
       </c>
       <c r="F118" t="n">
-        <v>22892.61158442801</v>
+        <v>25.40660919204317</v>
       </c>
     </row>
     <row r="119">
@@ -3041,7 +3041,7 @@
         <v>851</v>
       </c>
       <c r="F119" t="n">
-        <v>20801.76910456653</v>
+        <v>27.29138277106923</v>
       </c>
     </row>
     <row r="120">
@@ -3063,7 +3063,7 @@
         <v>1021</v>
       </c>
       <c r="F120" t="n">
-        <v>20622.78867769133</v>
+        <v>18.35676498860554</v>
       </c>
     </row>
     <row r="121">
@@ -3085,7 +3085,7 @@
         <v>1108</v>
       </c>
       <c r="F121" t="n">
-        <v>23252.53961012049</v>
+        <v>25.78933405729632</v>
       </c>
     </row>
   </sheetData>

</xml_diff>